<commit_message>
Added historic PE and EPS to FinancialData table (#8)
* test

* fine tune

* Updated doc
</commit_message>
<xml_diff>
--- a/DataColorTreshold.xlsx
+++ b/DataColorTreshold.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspaces\pinescript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9769E6-AA25-44A1-BFD5-DD97BC821C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04450E0C-09B5-4493-84E4-C84BADA038DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="64">
   <si>
     <t>Data Published Freq</t>
   </si>
@@ -54,12 +54,6 @@
     <t>P/E</t>
   </si>
   <si>
-    <t>&lt;= 25</t>
-  </si>
-  <si>
-    <t>&lt;0 OR &gt;25</t>
-  </si>
-  <si>
     <t>current market price divided by EPS</t>
   </si>
   <si>
@@ -214,6 +208,15 @@
   </si>
   <si>
     <t>New value (Feb 09 2026)</t>
+  </si>
+  <si>
+    <t>&gt;0 AND &lt;= 10 last years average</t>
+  </si>
+  <si>
+    <t>&lt;=0  OR &gt; 20%+ 10 last years average</t>
+  </si>
+  <si>
+    <t>&lt;= 10 last year average AND &lt;= 20%+ 10 last years average</t>
   </si>
 </sst>
 </file>
@@ -251,7 +254,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -282,6 +285,18 @@
         <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFC0C0C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -295,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -312,6 +327,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,9 +594,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31" customWidth="1"/>
+    <col min="5" max="5" width="53.5703125" customWidth="1"/>
+    <col min="6" max="6" width="36.7109375" customWidth="1"/>
     <col min="7" max="7" width="20" style="1" customWidth="1"/>
     <col min="8" max="8" width="66.42578125" customWidth="1"/>
     <col min="9" max="9" width="24.7109375" style="1" customWidth="1"/>
@@ -593,7 +610,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="3:9" x14ac:dyDescent="0.25">
@@ -621,47 +638,53 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
         <v>9</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="H5" t="s">
         <v>14</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="G6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="H6" t="s">
         <v>19</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>6</v>
@@ -669,22 +692,22 @@
     </row>
     <row r="7" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="G7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" t="s">
         <v>24</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>26</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>6</v>
@@ -692,33 +715,33 @@
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="H8" t="s">
         <v>28</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" t="s">
         <v>31</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" t="s">
-        <v>33</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>6</v>
@@ -726,119 +749,119 @@
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="F10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" t="s">
-        <v>38</v>
-      </c>
       <c r="I10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="F11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>42</v>
-      </c>
       <c r="I11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" t="s">
         <v>43</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="13" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" t="s">
         <v>44</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="15" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="F15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="G15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" t="s">
         <v>50</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" t="s">
-        <v>52</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>6</v>
@@ -846,22 +869,22 @@
     </row>
     <row r="16" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="F16" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="G16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" t="s">
         <v>55</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" t="s">
-        <v>57</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>6</v>
@@ -869,22 +892,22 @@
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" s="5" t="s">
+      <c r="G17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" t="s">
         <v>59</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" t="s">
-        <v>61</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>6</v>

</xml_diff>